<commit_message>
Update CDA EN/PN to FHIR HumanName mappings c01545caa11c5b77817b7dc131f2e9dc29b8f8e2
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaENPNToHumanNameConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaENPNToHumanNameConceptMap.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="66">
   <si>
     <t>Property</t>
   </si>
@@ -25,7 +25,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaNamesToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaENPNToHumanNameConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T12:48:49+00:00</t>
+    <t>2026-07-22T12:56:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -115,7 +115,10 @@
     <t>http://hl7.org/fhir/StructureDefinition/HumanName|4.0.1</t>
   </si>
   <si>
-    <t>EN.family</t>
+    <t>EN.item.family</t>
+  </si>
+  <si>
+    <t>Family</t>
   </si>
   <si>
     <t>equivalent</t>
@@ -124,25 +127,49 @@
     <t>HumanName.family</t>
   </si>
   <si>
-    <t>EN.given</t>
+    <t>Family name (often called 'Surname')</t>
+  </si>
+  <si>
+    <t>EN.item.given</t>
+  </si>
+  <si>
+    <t>Given</t>
   </si>
   <si>
     <t>HumanName.given</t>
   </si>
   <si>
-    <t>EN.prefix</t>
+    <t>Given names (not always 'first'). Includes middle names</t>
+  </si>
+  <si>
+    <t>EN.item.prefix</t>
+  </si>
+  <si>
+    <t>Prefix</t>
   </si>
   <si>
     <t>HumanName.prefix</t>
   </si>
   <si>
-    <t>EN.suffix</t>
+    <t>Parts that come before the name</t>
+  </si>
+  <si>
+    <t>EN.item.suffix</t>
+  </si>
+  <si>
+    <t>Suffix</t>
   </si>
   <si>
     <t>HumanName.suffix</t>
   </si>
   <si>
-    <t>EN.xmlText</t>
+    <t>Parts that come after the name</t>
+  </si>
+  <si>
+    <t>EN.item.xmlText</t>
+  </si>
+  <si>
+    <t>Allows for mixed text content</t>
   </si>
   <si>
     <t>related-to</t>
@@ -151,28 +178,37 @@
     <t>HumanName.text</t>
   </si>
   <si>
+    <t>Text representation of the full name</t>
+  </si>
+  <si>
     <t>EN.validTime</t>
   </si>
   <si>
+    <t>Valid Time</t>
+  </si>
+  <si>
     <t>HumanName.period</t>
   </si>
   <si>
+    <t>Time period when name was/is in use</t>
+  </si>
+  <si>
     <t>http://hl7.org/cda/stds/core/StructureDefinition/PN|2.0.0-sd</t>
   </si>
   <si>
-    <t>PN.family</t>
-  </si>
-  <si>
-    <t>PN.given</t>
-  </si>
-  <si>
-    <t>PN.prefix</t>
-  </si>
-  <si>
-    <t>PN.suffix</t>
-  </si>
-  <si>
-    <t>PN.xmlText</t>
+    <t>PN.item.family</t>
+  </si>
+  <si>
+    <t>PN.item.given</t>
+  </si>
+  <si>
+    <t>PN.item.prefix</t>
+  </si>
+  <si>
+    <t>PN.item.suffix</t>
+  </si>
+  <si>
+    <t>PN.item.xmlText</t>
   </si>
   <si>
     <t>PN.validTime</t>
@@ -473,101 +509,101 @@
         <v>33</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s" s="2">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -599,7 +635,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -616,104 +652,104 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s" s="2">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s" s="2">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
+        <v>64</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s" s="2">
         <v>52</v>
       </c>
-      <c r="B7" t="s" s="2">
-        <v>52</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>43</v>
-      </c>
       <c r="D7" t="s" s="2">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>